<commit_message>
Dedupliceer negatieve locaties + nieuwe Eigen Merk BE varianten
- _parse_locations ontdubbelt nu locatie-tuples (zelfde ID/naam wordt maar 1x toegevoegd)
- Eigen Merk BE variants.xlsx bijgewerkt: Schouwveger lange variant nu 'Uw Erkende Schouwveger'

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/branch_files/Schoorsteenveger/Eigen merk/BE/variants.xlsx
+++ b/branch_files/Schoorsteenveger/Eigen merk/BE/variants.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\menno\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{511EA976-38E4-4E3E-A595-205C7C3AFABC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC1FC7A2-D461-48B5-B529-CBC745F6C12C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -167,10 +167,10 @@
     <t>Schoorsteenveger In De Buurt</t>
   </si>
   <si>
-    <t>Schouwveger In De Buurt</t>
-  </si>
-  <si>
     <t>In [Plaats]</t>
+  </si>
+  <si>
+    <t>Uw Erkende Schouwveger</t>
   </si>
 </sst>
 </file>
@@ -563,7 +563,7 @@
         <v>13</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>14</v>
@@ -722,7 +722,7 @@
         <v>35</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E13" s="5" t="s">
         <v>33</v>

</xml_diff>